<commit_message>
phase5: Apify→Firestore pipeline rebuild + cron trigger
- Add app/api/cron/scrape/route.ts: triggers Apify runs on schedule
- Fix startApifyRun: payloadTemplate with explicit datasetId, SUCCEEDED-only events
- Fix webhook handler: robust unsubstituted-template guard using includes('{{')
- Add CRON_SECRET to apphosting.yaml
- Post creation UI updates (PostScreen, PostPage, App.tsx)
- Gemini service and actions improvements

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FacebookGroups.xlsx
+++ b/FacebookGroups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/750b1f02a83a37d5/Projects/subhub (27.01.26)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="8_{5360561F-91B4-4B51-823D-E64B5AF1C9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CB636C1-73D8-4F0B-BBE4-2EC9D274260F}"/>
+  <xr:revisionPtr revIDLastSave="93" documentId="8_{5360561F-91B4-4B51-823D-E64B5AF1C9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1711B065-9A34-4B64-8584-639141A3FA58}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{BD637D88-55B9-47DD-8CF9-D8C1F2F9154D}"/>
   </bookViews>
@@ -17,10 +17,9 @@
     <sheet name="Actor - Full List" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Actor - Partial List'!$A$1:$E$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Actor - Partial List'!$A$1:$F$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="74">
   <si>
     <t>Facebook Group URL</t>
   </si>
@@ -257,6 +256,12 @@
   </si>
   <si>
     <t>Comments</t>
+  </si>
+  <si>
+    <t>Israel</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/1253641912158395</t>
   </si>
 </sst>
 </file>
@@ -648,533 +653,577 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED79D08-BA05-4440-90F8-6ED3B9BF540C}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="60.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.69921875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="2"/>
+    <col min="3" max="3" width="21.69921875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="1"/>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="D8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="D25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C31" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C32" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C33" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="D36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="D37" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E33" xr:uid="{5ED79D08-BA05-4440-90F8-6ED3B9BF540C}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="High"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="A1:F37" xr:uid="{5ED79D08-BA05-4440-90F8-6ED3B9BF540C}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F37">
+      <sortCondition ref="B1:B37"/>
+    </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="A23" r:id="rId1" xr:uid="{4E8F285A-E7A5-46FF-9EF7-4AD23DCA286D}"/>
-    <hyperlink ref="A13" r:id="rId2" xr:uid="{25D4579C-E55B-45BE-A2CB-B519B9DB95D2}"/>
-    <hyperlink ref="A25" r:id="rId3" xr:uid="{092423C6-1C13-44EE-8228-AFE0A31A6239}"/>
-    <hyperlink ref="A42" r:id="rId4" xr:uid="{A589DF09-AC48-4F3A-B3FE-58445B3F55A5}"/>
-    <hyperlink ref="A44" r:id="rId5" xr:uid="{886A6581-1088-436C-B5E4-09FA3CAADC77}"/>
+    <hyperlink ref="A27" r:id="rId1" xr:uid="{4E8F285A-E7A5-46FF-9EF7-4AD23DCA286D}"/>
+    <hyperlink ref="A14" r:id="rId2" xr:uid="{25D4579C-E55B-45BE-A2CB-B519B9DB95D2}"/>
+    <hyperlink ref="A29" r:id="rId3" xr:uid="{092423C6-1C13-44EE-8228-AFE0A31A6239}"/>
+    <hyperlink ref="A46" r:id="rId4" xr:uid="{A589DF09-AC48-4F3A-B3FE-58445B3F55A5}"/>
+    <hyperlink ref="A48" r:id="rId5" xr:uid="{886A6581-1088-436C-B5E4-09FA3CAADC77}"/>
+    <hyperlink ref="A30" r:id="rId6" xr:uid="{11AD953C-37C4-49E6-A1A0-60E242E648DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: onlyWithPrice filter, time-ago badges, carousel click fixes, language sync
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/FacebookGroups.xlsx
+++ b/FacebookGroups.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/750b1f02a83a37d5/Projects/subhub (27.01.26)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="8_{5360561F-91B4-4B51-823D-E64B5AF1C9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1711B065-9A34-4B64-8584-639141A3FA58}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{5360561F-91B4-4B51-823D-E64B5AF1C9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1396966E-ED39-4099-92EB-9FB525B40481}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{BD637D88-55B9-47DD-8CF9-D8C1F2F9154D}"/>
+    <workbookView minimized="1" xWindow="1536" yWindow="1236" windowWidth="21600" windowHeight="11100" xr2:uid="{BD637D88-55B9-47DD-8CF9-D8C1F2F9154D}"/>
   </bookViews>
   <sheets>
     <sheet name="Actor - Partial List" sheetId="1" r:id="rId1"/>
@@ -653,17 +653,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ED79D08-BA05-4440-90F8-6ED3B9BF540C}">
-  <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="60.09765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.69921875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.69921875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="60.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.75" style="2" customWidth="1"/>
     <col min="4" max="4" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -681,7 +681,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
@@ -695,7 +695,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -709,7 +709,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>47</v>
       </c>
@@ -723,7 +723,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -737,7 +737,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>60</v>
       </c>
@@ -751,7 +751,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -765,7 +765,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -779,7 +779,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>51</v>
       </c>
@@ -793,7 +793,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
@@ -807,7 +807,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -821,7 +821,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
@@ -835,7 +835,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>21</v>
       </c>
@@ -849,7 +849,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
@@ -863,7 +863,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>49</v>
       </c>
@@ -877,7 +877,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>37</v>
       </c>
@@ -891,7 +891,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>45</v>
       </c>
@@ -905,7 +905,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>43</v>
       </c>
@@ -919,7 +919,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>27</v>
       </c>
@@ -933,7 +933,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>54</v>
       </c>
@@ -947,7 +947,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>3</v>
       </c>
@@ -961,7 +961,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>6</v>
       </c>
@@ -975,7 +975,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
@@ -989,7 +989,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
@@ -1003,7 +1003,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>62</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>12</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>7</v>
       </c>
@@ -1065,7 +1065,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>69</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>73</v>
       </c>
@@ -1102,17 +1102,17 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C31" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C33" s="2" t="s">
         <v>72</v>
       </c>
@@ -1120,7 +1120,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>52</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>56</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>39</v>
       </c>
@@ -1162,7 +1162,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>58</v>
       </c>
@@ -1176,38 +1176,38 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1221,8 +1221,8 @@
     <hyperlink ref="A27" r:id="rId1" xr:uid="{4E8F285A-E7A5-46FF-9EF7-4AD23DCA286D}"/>
     <hyperlink ref="A14" r:id="rId2" xr:uid="{25D4579C-E55B-45BE-A2CB-B519B9DB95D2}"/>
     <hyperlink ref="A29" r:id="rId3" xr:uid="{092423C6-1C13-44EE-8228-AFE0A31A6239}"/>
-    <hyperlink ref="A46" r:id="rId4" xr:uid="{A589DF09-AC48-4F3A-B3FE-58445B3F55A5}"/>
-    <hyperlink ref="A48" r:id="rId5" xr:uid="{886A6581-1088-436C-B5E4-09FA3CAADC77}"/>
+    <hyperlink ref="A38" r:id="rId4" xr:uid="{A589DF09-AC48-4F3A-B3FE-58445B3F55A5}"/>
+    <hyperlink ref="A40" r:id="rId5" xr:uid="{886A6581-1088-436C-B5E4-09FA3CAADC77}"/>
     <hyperlink ref="A30" r:id="rId6" xr:uid="{11AD953C-37C4-49E6-A1A0-60E242E648DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1232,172 +1232,172 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0D3B185-8379-47CB-9F9D-47CA5F45BE20}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="60.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="60.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>62</v>
       </c>

</xml_diff>